<commit_message>
Refactor LBO model builder for readability
Split the single flat script into one function per sheet, replace ~40
loose ROW_* globals with named per-sheet row dicts (a/su/om/fcf/ds),
and add a module docstring covering the sheet dependency order and two
non-obvious design choices: beginning-balance interest (avoids a
circular reference) and the fixed forecast-year columns. Also removes
two dead-code spots where a placeholder formula was written then
silently overwritten. Verified output is numerically identical to the
prior version (same S&U check, leverage, MOIC, IRR).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LBO_Model.xlsx
+++ b/LBO_Model.xlsx
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="B3" s="15">
-        <f>Assumptions!$B$5</f>
+        <f>'Assumptions'!$B$5</f>
         <v/>
       </c>
       <c r="C3" s="15">
@@ -1043,27 +1043,27 @@
         </is>
       </c>
       <c r="B4" s="10">
-        <f>Assumptions!$B$13</f>
+        <f>'Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="C4" s="10">
-        <f>B4*(1+Assumptions!$B$14)</f>
+        <f>B4*(1+'Assumptions'!$B$14)</f>
         <v/>
       </c>
       <c r="D4" s="10">
-        <f>C4*(1+Assumptions!$B$14)</f>
+        <f>C4*(1+'Assumptions'!$B$14)</f>
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>D4*(1+Assumptions!$B$14)</f>
+        <f>D4*(1+'Assumptions'!$B$14)</f>
         <v/>
       </c>
       <c r="F4" s="10">
-        <f>E4*(1+Assumptions!$B$14)</f>
+        <f>E4*(1+'Assumptions'!$B$14)</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>F4*(1+Assumptions!$B$14)</f>
+        <f>F4*(1+'Assumptions'!$B$14)</f>
         <v/>
       </c>
     </row>
@@ -1102,27 +1102,27 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>Assumptions!$B$15</f>
+        <f>'Assumptions'!$B$15</f>
         <v/>
       </c>
       <c r="C6" s="16">
-        <f>B6+Assumptions!$B$16</f>
+        <f>B6+'Assumptions'!$B$16</f>
         <v/>
       </c>
       <c r="D6" s="16">
-        <f>C6+Assumptions!$B$16</f>
+        <f>C6+'Assumptions'!$B$16</f>
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>D6+Assumptions!$B$16</f>
+        <f>D6+'Assumptions'!$B$16</f>
         <v/>
       </c>
       <c r="F6" s="16">
-        <f>E6+Assumptions!$B$16</f>
+        <f>E6+'Assumptions'!$B$16</f>
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>F6+Assumptions!$B$16</f>
+        <f>F6+'Assumptions'!$B$16</f>
         <v/>
       </c>
     </row>
@@ -1164,27 +1164,27 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>-B4*Assumptions!$B$17</f>
+        <f>-B4*'Assumptions'!$B$17</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>-C4*Assumptions!$B$17</f>
+        <f>-C4*'Assumptions'!$B$17</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>-D4*Assumptions!$B$17</f>
+        <f>-D4*'Assumptions'!$B$17</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>-E4*Assumptions!$B$17</f>
+        <f>-E4*'Assumptions'!$B$17</f>
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>-F4*Assumptions!$B$17</f>
+        <f>-F4*'Assumptions'!$B$17</f>
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>-G4*Assumptions!$B$17</f>
+        <f>-G4*'Assumptions'!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1287,27 +1287,27 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>-MAX(B11,0)*Assumptions!$B$20</f>
+        <f>-MAX(B11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>-MAX(C11,0)*Assumptions!$B$20</f>
+        <f>-MAX(C11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>-MAX(D11,0)*Assumptions!$B$20</f>
+        <f>-MAX(D11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
       <c r="E12" s="11">
-        <f>-MAX(E11,0)*Assumptions!$B$20</f>
+        <f>-MAX(E11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
       <c r="F12" s="11">
-        <f>-MAX(F11,0)*Assumptions!$B$20</f>
+        <f>-MAX(F11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
       <c r="G12" s="11">
-        <f>-MAX(G11,0)*Assumptions!$B$20</f>
+        <f>-MAX(G11,0)*'Assumptions'!$B$20</f>
         <v/>
       </c>
     </row>
@@ -1476,23 +1476,23 @@
         <v>0</v>
       </c>
       <c r="C6" s="11">
-        <f>-'Operating Model'!C4*Assumptions!$B$18</f>
+        <f>-'Operating Model'!C4*'Assumptions'!$B$18</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>-'Operating Model'!D4*Assumptions!$B$18</f>
+        <f>-'Operating Model'!D4*'Assumptions'!$B$18</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>-'Operating Model'!E4*Assumptions!$B$18</f>
+        <f>-'Operating Model'!E4*'Assumptions'!$B$18</f>
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>-'Operating Model'!F4*Assumptions!$B$18</f>
+        <f>-'Operating Model'!F4*'Assumptions'!$B$18</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>-'Operating Model'!G4*Assumptions!$B$18</f>
+        <f>-'Operating Model'!G4*'Assumptions'!$B$18</f>
         <v/>
       </c>
     </row>
@@ -1506,23 +1506,23 @@
         <v>0</v>
       </c>
       <c r="C7" s="11">
-        <f>-('Operating Model'!C4-'Operating Model'!B4)*Assumptions!$B$19</f>
+        <f>-('Operating Model'!C4-'Operating Model'!B4)*'Assumptions'!$B$19</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>-('Operating Model'!D4-'Operating Model'!C4)*Assumptions!$B$19</f>
+        <f>-('Operating Model'!D4-'Operating Model'!C4)*'Assumptions'!$B$19</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>-('Operating Model'!E4-'Operating Model'!D4)*Assumptions!$B$19</f>
+        <f>-('Operating Model'!E4-'Operating Model'!D4)*'Assumptions'!$B$19</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>-('Operating Model'!F4-'Operating Model'!E4)*Assumptions!$B$19</f>
+        <f>-('Operating Model'!F4-'Operating Model'!E4)*'Assumptions'!$B$19</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>-('Operating Model'!G4-'Operating Model'!F4)*Assumptions!$B$19</f>
+        <f>-('Operating Model'!G4-'Operating Model'!F4)*'Assumptions'!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1691,23 +1691,23 @@
         <v>0</v>
       </c>
       <c r="C7" s="11">
-        <f>MAX(C5+C6,0)*Assumptions!$B$30</f>
+        <f>MAX(C5+C6,0)*'Assumptions'!$B$30</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>MAX(D5+D6,0)*Assumptions!$B$30</f>
+        <f>MAX(D5+D6,0)*'Assumptions'!$B$30</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>MAX(E5+E6,0)*Assumptions!$B$30</f>
+        <f>MAX(E5+E6,0)*'Assumptions'!$B$30</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>MAX(F5+F6,0)*Assumptions!$B$30</f>
+        <f>MAX(F5+F6,0)*'Assumptions'!$B$30</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>MAX(G5+G6,0)*Assumptions!$B$30</f>
+        <f>MAX(G5+G6,0)*'Assumptions'!$B$30</f>
         <v/>
       </c>
     </row>
@@ -1758,23 +1758,23 @@
         <v>0</v>
       </c>
       <c r="C11" s="11">
-        <f>-MIN('Sources &amp; Uses'!$B$12*Assumptions!$B$25,C10)</f>
+        <f>-MIN('Sources &amp; Uses'!$B$12*'Assumptions'!$B$25,C10)</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>-MIN('Sources &amp; Uses'!$B$12*Assumptions!$B$25,D10)</f>
+        <f>-MIN('Sources &amp; Uses'!$B$12*'Assumptions'!$B$25,D10)</f>
         <v/>
       </c>
       <c r="E11" s="11">
-        <f>-MIN('Sources &amp; Uses'!$B$12*Assumptions!$B$25,E10)</f>
+        <f>-MIN('Sources &amp; Uses'!$B$12*'Assumptions'!$B$25,E10)</f>
         <v/>
       </c>
       <c r="F11" s="11">
-        <f>-MIN('Sources &amp; Uses'!$B$12*Assumptions!$B$25,F10)</f>
+        <f>-MIN('Sources &amp; Uses'!$B$12*'Assumptions'!$B$25,F10)</f>
         <v/>
       </c>
       <c r="G11" s="11">
-        <f>-MIN('Sources &amp; Uses'!$B$12*Assumptions!$B$25,G10)</f>
+        <f>-MIN('Sources &amp; Uses'!$B$12*'Assumptions'!$B$25,G10)</f>
         <v/>
       </c>
     </row>
@@ -1849,23 +1849,23 @@
         <v>0</v>
       </c>
       <c r="C14" s="11">
-        <f>C10*Assumptions!$B$24</f>
+        <f>C10*'Assumptions'!$B$24</f>
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>D10*Assumptions!$B$24</f>
+        <f>D10*'Assumptions'!$B$24</f>
         <v/>
       </c>
       <c r="E14" s="11">
-        <f>E10*Assumptions!$B$24</f>
+        <f>E10*'Assumptions'!$B$24</f>
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>F10*Assumptions!$B$24</f>
+        <f>F10*'Assumptions'!$B$24</f>
         <v/>
       </c>
       <c r="G14" s="11">
-        <f>G10*Assumptions!$B$24</f>
+        <f>G10*'Assumptions'!$B$24</f>
         <v/>
       </c>
     </row>
@@ -1977,23 +1977,23 @@
         <v>0</v>
       </c>
       <c r="C20" s="11">
-        <f>C17*Assumptions!$B$27</f>
+        <f>C17*'Assumptions'!$B$27</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>D17*Assumptions!$B$27</f>
+        <f>D17*'Assumptions'!$B$27</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>E17*Assumptions!$B$27</f>
+        <f>E17*'Assumptions'!$B$27</f>
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>F17*Assumptions!$B$27</f>
+        <f>F17*'Assumptions'!$B$27</f>
         <v/>
       </c>
       <c r="G20" s="11">
-        <f>G17*Assumptions!$B$27</f>
+        <f>G17*'Assumptions'!$B$27</f>
         <v/>
       </c>
     </row>
@@ -2106,23 +2106,23 @@
         <v>0</v>
       </c>
       <c r="C26" s="11">
-        <f>C23*Assumptions!$B$28</f>
+        <f>C23*'Assumptions'!$B$28</f>
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>D23*Assumptions!$B$28</f>
+        <f>D23*'Assumptions'!$B$28</f>
         <v/>
       </c>
       <c r="E26" s="11">
-        <f>E23*Assumptions!$B$28</f>
+        <f>E23*'Assumptions'!$B$28</f>
         <v/>
       </c>
       <c r="F26" s="11">
-        <f>F23*Assumptions!$B$28</f>
+        <f>F23*'Assumptions'!$B$28</f>
         <v/>
       </c>
       <c r="G26" s="11">
-        <f>G23*Assumptions!$B$28</f>
+        <f>G23*'Assumptions'!$B$28</f>
         <v/>
       </c>
     </row>
@@ -2195,27 +2195,27 @@
         </is>
       </c>
       <c r="B30" s="11">
-        <f>Assumptions!$B$29</f>
+        <f>'Assumptions'!$B$29</f>
         <v/>
       </c>
       <c r="C30" s="11">
-        <f>B30+MAX(C5+C6+C12+C18,0)*(1-Assumptions!$B$30)</f>
+        <f>B30+MAX(C5+C6+C12+C18,0)*(1-'Assumptions'!$B$30)</f>
         <v/>
       </c>
       <c r="D30" s="11">
-        <f>C30+MAX(D5+D6+D12+D18,0)*(1-Assumptions!$B$30)</f>
+        <f>C30+MAX(D5+D6+D12+D18,0)*(1-'Assumptions'!$B$30)</f>
         <v/>
       </c>
       <c r="E30" s="11">
-        <f>D30+MAX(E5+E6+E12+E18,0)*(1-Assumptions!$B$30)</f>
+        <f>D30+MAX(E5+E6+E12+E18,0)*(1-'Assumptions'!$B$30)</f>
         <v/>
       </c>
       <c r="F30" s="11">
-        <f>E30+MAX(F5+F6+F12+F18,0)*(1-Assumptions!$B$30)</f>
+        <f>E30+MAX(F5+F6+F12+F18,0)*(1-'Assumptions'!$B$30)</f>
         <v/>
       </c>
       <c r="G30" s="11">
-        <f>F30+MAX(G5+G6+G12+G18,0)*(1-Assumptions!$B$30)</f>
+        <f>F30+MAX(G5+G6+G12+G18,0)*(1-'Assumptions'!$B$30)</f>
         <v/>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="B5" s="14">
-        <f>Assumptions!$B$8</f>
+        <f>'Assumptions'!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>B4*Assumptions!$B$8</f>
+        <f>B4*'Assumptions'!$B$8</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>'Sources &amp; Uses'!B$17</f>
+        <f>'Sources &amp; Uses'!$B$17</f>
         <v/>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>B8*(1-Assumptions!$B$31)</f>
+        <f>B8*(1-'Assumptions'!$B$31)</f>
         <v/>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="B13" s="17">
-        <f>Assumptions!$B$6</f>
+        <f>'Assumptions'!$B$6</f>
         <v/>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Note: exit assumed at end of Year 5 (col G). Adjust Hold Period + column refs on this tab if you change the hold period.</t>
+          <t>Note: exit assumed at end of Year 5 (col G). Change FORECAST_YEARS in the script if you want a different hold length.</t>
         </is>
       </c>
     </row>

</xml_diff>